<commit_message>
Fixed the non-GAAP items in WDC model and added info about other income/expenses in the instructions
</commit_message>
<xml_diff>
--- a/_Instructions and Theory/9. Statement and Data Notes.xlsx
+++ b/_Instructions and Theory/9. Statement and Data Notes.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/_Instructions and Theory/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062241AD-2716-2444-888B-6CF5FC6E2580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4561C1C2-0AB7-8C4E-940F-FAB3430A28B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="100" windowWidth="25440" windowHeight="13540" activeTab="2" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="80" yWindow="100" windowWidth="25440" windowHeight="13540" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Misc" sheetId="1" r:id="rId1"/>
-    <sheet name="Balance sheet" sheetId="2" r:id="rId2"/>
-    <sheet name="Cash flow statement" sheetId="3" r:id="rId3"/>
+    <sheet name="Income statement" sheetId="5" r:id="rId1"/>
+    <sheet name="Misc" sheetId="1" r:id="rId2"/>
+    <sheet name="Balance sheet" sheetId="2" r:id="rId3"/>
+    <sheet name="Cash flow statement" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Debt is formed from finance and operating leases</t>
   </si>
@@ -131,6 +133,27 @@
   </si>
   <si>
     <t>Operating net working capital</t>
+  </si>
+  <si>
+    <t>In other income we will sometimes have one-time items like sale of part of a business which we have to take out</t>
+  </si>
+  <si>
+    <t>Sales of assets are also considered one off which should be removed</t>
+  </si>
+  <si>
+    <t>Debt to equity exchanges or equity to equity exchanges should also be removed</t>
+  </si>
+  <si>
+    <t>In such cases we have to find the non-GAAP tax rate in the company documents like presentation/ press release, 10-K/10-Q</t>
+  </si>
+  <si>
+    <t>We have to recalculate the pre tax income,  taxes paid with that rate, then the net income and EPS</t>
+  </si>
+  <si>
+    <t>Other income/expenses</t>
+  </si>
+  <si>
+    <t>We can also find the non-GAAP taxes paid usually in the press release under the 3 GAAP statements which we can use</t>
   </si>
 </sst>
 </file>
@@ -587,6 +610,64 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70674F52-2140-9546-92C8-89BE0BE5143F}">
+  <dimension ref="A2:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="7.5" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{825B172E-7ADE-4B4A-B533-F037BCFCDCB0}">
   <dimension ref="A2:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -753,7 +834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{814D76A1-7D08-704B-BAAB-375DB2AC65BF}">
   <dimension ref="A2:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -820,7 +901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B52D245-5CCA-F14A-92B0-79B3A2EC7B79}">
   <dimension ref="A2:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -851,4 +932,13 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBA6ADA4-129A-8C41-9554-C31E5219B124}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>